<commit_message>
add info to TPSR Template dan merubah L0 dst ke text yang sesuai
</commit_message>
<xml_diff>
--- a/public/TPSR_template.xlsx
+++ b/public/TPSR_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\d\magang\simagang\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\web-tpsr\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A3F5B5-6148-4B1A-8C59-AECF5834B5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C944E3-595E-4D34-A4E4-2973BE197A23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="42">
   <si>
     <t>Nama Siswa</t>
   </si>
@@ -155,15 +155,39 @@
     <t>5-D</t>
   </si>
   <si>
-    <t>NB: ini hanyalah template, isi dengan data yang anda inginkan</t>
+    <t>NB:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dokumen ini hanya merupakan template. Silakan isi setiap field dengan data yang sesuai dengan kebutuhan. Untuk field Kelas, harap menggantinya dengan nama kelas yang sebenarnya berdasarkan data yang akan diinput. Apabila data kelas yang diinput sudah tersedia dalam sistem, maka data siswa dan penilaiannya akan ditambahkan ke kelas tersebut. Jika data kelas belum tersedia, sistem akan secara otomatis membuat kelas baru beserta data siswa dan penilaiannya sesuai dengan informasi yang diberikan. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mohon untuk tidak mengubah struktur template ini agar proses impor data dapat berjalan dengan baik.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -209,24 +233,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:CC13"/>
+  <dimension ref="A2:CC17"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -540,132 +571,132 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:81" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:81" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="1" t="s">
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="AB3" s="2"/>
-      <c r="AC3" s="2"/>
-      <c r="AD3" s="2"/>
-      <c r="AE3" s="2"/>
-      <c r="AF3" s="1" t="s">
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="AG3" s="2"/>
-      <c r="AH3" s="2"/>
-      <c r="AI3" s="2"/>
-      <c r="AJ3" s="2"/>
-      <c r="AK3" s="1" t="s">
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="AL3" s="2"/>
-      <c r="AM3" s="2"/>
-      <c r="AN3" s="2"/>
-      <c r="AO3" s="2"/>
-      <c r="AP3" s="1" t="s">
+      <c r="AL3" s="3"/>
+      <c r="AM3" s="3"/>
+      <c r="AN3" s="3"/>
+      <c r="AO3" s="3"/>
+      <c r="AP3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="AQ3" s="2"/>
-      <c r="AR3" s="2"/>
-      <c r="AS3" s="2"/>
-      <c r="AT3" s="2"/>
-      <c r="AU3" s="1" t="s">
+      <c r="AQ3" s="3"/>
+      <c r="AR3" s="3"/>
+      <c r="AS3" s="3"/>
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="AV3" s="2"/>
-      <c r="AW3" s="2"/>
-      <c r="AX3" s="2"/>
-      <c r="AY3" s="2"/>
-      <c r="AZ3" s="1" t="s">
+      <c r="AV3" s="3"/>
+      <c r="AW3" s="3"/>
+      <c r="AX3" s="3"/>
+      <c r="AY3" s="3"/>
+      <c r="AZ3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="BA3" s="2"/>
-      <c r="BB3" s="2"/>
-      <c r="BC3" s="2"/>
-      <c r="BD3" s="2"/>
-      <c r="BE3" s="1" t="s">
+      <c r="BA3" s="3"/>
+      <c r="BB3" s="3"/>
+      <c r="BC3" s="3"/>
+      <c r="BD3" s="3"/>
+      <c r="BE3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="BF3" s="2"/>
-      <c r="BG3" s="2"/>
-      <c r="BH3" s="2"/>
-      <c r="BI3" s="2"/>
-      <c r="BJ3" s="1" t="s">
+      <c r="BF3" s="3"/>
+      <c r="BG3" s="3"/>
+      <c r="BH3" s="3"/>
+      <c r="BI3" s="3"/>
+      <c r="BJ3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="BK3" s="2"/>
-      <c r="BL3" s="2"/>
-      <c r="BM3" s="2"/>
-      <c r="BN3" s="2"/>
-      <c r="BO3" s="1" t="s">
+      <c r="BK3" s="3"/>
+      <c r="BL3" s="3"/>
+      <c r="BM3" s="3"/>
+      <c r="BN3" s="3"/>
+      <c r="BO3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="BP3" s="2"/>
-      <c r="BQ3" s="2"/>
-      <c r="BR3" s="2"/>
-      <c r="BS3" s="2"/>
-      <c r="BT3" s="1" t="s">
+      <c r="BP3" s="3"/>
+      <c r="BQ3" s="3"/>
+      <c r="BR3" s="3"/>
+      <c r="BS3" s="3"/>
+      <c r="BT3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BU3" s="2"/>
-      <c r="BV3" s="2"/>
-      <c r="BW3" s="2"/>
-      <c r="BX3" s="2"/>
-      <c r="BY3" s="1" t="s">
+      <c r="BU3" s="3"/>
+      <c r="BV3" s="3"/>
+      <c r="BW3" s="3"/>
+      <c r="BX3" s="3"/>
+      <c r="BY3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="BZ3" s="2"/>
-      <c r="CA3" s="2"/>
-      <c r="CB3" s="2"/>
-      <c r="CC3" s="2"/>
+      <c r="BZ3" s="3"/>
+      <c r="CA3" s="3"/>
+      <c r="CB3" s="3"/>
+      <c r="CC3" s="3"/>
     </row>
     <row r="4" spans="1:81" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
       <c r="B4" t="s">
         <v>17</v>
       </c>
@@ -2132,13 +2163,85 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:81" x14ac:dyDescent="0.3">
-      <c r="D13" t="s">
+    <row r="13" spans="1:81" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="10" t="s">
         <v>40</v>
       </c>
+      <c r="D13" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+    </row>
+    <row r="14" spans="1:81" x14ac:dyDescent="0.3">
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+    </row>
+    <row r="15" spans="1:81" x14ac:dyDescent="0.3">
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+    </row>
+    <row r="16" spans="1:81" x14ac:dyDescent="0.3">
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+    </row>
+    <row r="17" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="19">
+    <mergeCell ref="Q3:U3"/>
+    <mergeCell ref="C13:C17"/>
+    <mergeCell ref="D13:N17"/>
     <mergeCell ref="AF3:AJ3"/>
     <mergeCell ref="L3:P3"/>
     <mergeCell ref="AA3:AE3"/>
@@ -2155,7 +2258,6 @@
     <mergeCell ref="BE3:BI3"/>
     <mergeCell ref="BT3:BX3"/>
     <mergeCell ref="V3:Z3"/>
-    <mergeCell ref="Q3:U3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2170,204 +2272,204 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:161" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="W1" s="6"/>
-      <c r="X1" s="6"/>
-      <c r="Y1" s="6"/>
-      <c r="Z1" s="6"/>
-      <c r="AA1" s="6"/>
-      <c r="AB1" s="6"/>
-      <c r="AC1" s="6"/>
-      <c r="AD1" s="6"/>
-      <c r="AE1" s="6"/>
-      <c r="AF1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="AG1" s="2"/>
-      <c r="AH1" s="2"/>
-      <c r="AI1" s="2"/>
-      <c r="AJ1" s="2"/>
-      <c r="AK1" s="2"/>
-      <c r="AL1" s="2"/>
-      <c r="AM1" s="2"/>
-      <c r="AN1" s="2"/>
-      <c r="AO1" s="2"/>
-      <c r="AP1" s="1" t="s">
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="7"/>
+      <c r="V1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5"/>
+      <c r="AA1" s="5"/>
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="5"/>
+      <c r="AD1" s="5"/>
+      <c r="AE1" s="5"/>
+      <c r="AF1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="AG1" s="3"/>
+      <c r="AH1" s="3"/>
+      <c r="AI1" s="3"/>
+      <c r="AJ1" s="3"/>
+      <c r="AK1" s="3"/>
+      <c r="AL1" s="3"/>
+      <c r="AM1" s="3"/>
+      <c r="AN1" s="3"/>
+      <c r="AO1" s="3"/>
+      <c r="AP1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="AQ1" s="2"/>
-      <c r="AR1" s="2"/>
-      <c r="AS1" s="2"/>
-      <c r="AT1" s="2"/>
-      <c r="AU1" s="2"/>
-      <c r="AV1" s="2"/>
-      <c r="AW1" s="2"/>
-      <c r="AX1" s="2"/>
-      <c r="AY1" s="2"/>
-      <c r="AZ1" s="1" t="s">
+      <c r="AQ1" s="3"/>
+      <c r="AR1" s="3"/>
+      <c r="AS1" s="3"/>
+      <c r="AT1" s="3"/>
+      <c r="AU1" s="3"/>
+      <c r="AV1" s="3"/>
+      <c r="AW1" s="3"/>
+      <c r="AX1" s="3"/>
+      <c r="AY1" s="3"/>
+      <c r="AZ1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="BA1" s="2"/>
-      <c r="BB1" s="2"/>
-      <c r="BC1" s="2"/>
-      <c r="BD1" s="2"/>
-      <c r="BE1" s="2"/>
-      <c r="BF1" s="2"/>
-      <c r="BG1" s="2"/>
-      <c r="BH1" s="2"/>
-      <c r="BI1" s="2"/>
-      <c r="BJ1" s="1" t="s">
+      <c r="BA1" s="3"/>
+      <c r="BB1" s="3"/>
+      <c r="BC1" s="3"/>
+      <c r="BD1" s="3"/>
+      <c r="BE1" s="3"/>
+      <c r="BF1" s="3"/>
+      <c r="BG1" s="3"/>
+      <c r="BH1" s="3"/>
+      <c r="BI1" s="3"/>
+      <c r="BJ1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="BK1" s="2"/>
-      <c r="BL1" s="2"/>
-      <c r="BM1" s="2"/>
-      <c r="BN1" s="2"/>
-      <c r="BO1" s="2"/>
-      <c r="BP1" s="2"/>
-      <c r="BQ1" s="2"/>
-      <c r="BR1" s="2"/>
-      <c r="BS1" s="2"/>
-      <c r="BT1" s="1" t="s">
+      <c r="BK1" s="3"/>
+      <c r="BL1" s="3"/>
+      <c r="BM1" s="3"/>
+      <c r="BN1" s="3"/>
+      <c r="BO1" s="3"/>
+      <c r="BP1" s="3"/>
+      <c r="BQ1" s="3"/>
+      <c r="BR1" s="3"/>
+      <c r="BS1" s="3"/>
+      <c r="BT1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="BU1" s="2"/>
-      <c r="BV1" s="2"/>
-      <c r="BW1" s="2"/>
-      <c r="BX1" s="2"/>
-      <c r="BY1" s="2"/>
-      <c r="BZ1" s="2"/>
-      <c r="CA1" s="2"/>
-      <c r="CB1" s="2"/>
-      <c r="CC1" s="2"/>
-      <c r="CD1" s="1" t="s">
+      <c r="BU1" s="3"/>
+      <c r="BV1" s="3"/>
+      <c r="BW1" s="3"/>
+      <c r="BX1" s="3"/>
+      <c r="BY1" s="3"/>
+      <c r="BZ1" s="3"/>
+      <c r="CA1" s="3"/>
+      <c r="CB1" s="3"/>
+      <c r="CC1" s="3"/>
+      <c r="CD1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="CE1" s="2"/>
-      <c r="CF1" s="2"/>
-      <c r="CG1" s="2"/>
-      <c r="CH1" s="2"/>
-      <c r="CI1" s="2"/>
-      <c r="CJ1" s="2"/>
-      <c r="CK1" s="2"/>
-      <c r="CL1" s="2"/>
-      <c r="CM1" s="2"/>
-      <c r="CN1" s="1" t="s">
+      <c r="CE1" s="3"/>
+      <c r="CF1" s="3"/>
+      <c r="CG1" s="3"/>
+      <c r="CH1" s="3"/>
+      <c r="CI1" s="3"/>
+      <c r="CJ1" s="3"/>
+      <c r="CK1" s="3"/>
+      <c r="CL1" s="3"/>
+      <c r="CM1" s="3"/>
+      <c r="CN1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="CO1" s="2"/>
-      <c r="CP1" s="2"/>
-      <c r="CQ1" s="2"/>
-      <c r="CR1" s="2"/>
-      <c r="CS1" s="2"/>
-      <c r="CT1" s="2"/>
-      <c r="CU1" s="2"/>
-      <c r="CV1" s="2"/>
-      <c r="CW1" s="2"/>
-      <c r="CX1" s="1" t="s">
+      <c r="CO1" s="3"/>
+      <c r="CP1" s="3"/>
+      <c r="CQ1" s="3"/>
+      <c r="CR1" s="3"/>
+      <c r="CS1" s="3"/>
+      <c r="CT1" s="3"/>
+      <c r="CU1" s="3"/>
+      <c r="CV1" s="3"/>
+      <c r="CW1" s="3"/>
+      <c r="CX1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="CY1" s="2"/>
-      <c r="CZ1" s="2"/>
-      <c r="DA1" s="2"/>
-      <c r="DB1" s="2"/>
-      <c r="DC1" s="2"/>
-      <c r="DD1" s="2"/>
-      <c r="DE1" s="2"/>
-      <c r="DF1" s="2"/>
-      <c r="DG1" s="2"/>
-      <c r="DH1" s="1" t="s">
+      <c r="CY1" s="3"/>
+      <c r="CZ1" s="3"/>
+      <c r="DA1" s="3"/>
+      <c r="DB1" s="3"/>
+      <c r="DC1" s="3"/>
+      <c r="DD1" s="3"/>
+      <c r="DE1" s="3"/>
+      <c r="DF1" s="3"/>
+      <c r="DG1" s="3"/>
+      <c r="DH1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="DI1" s="2"/>
-      <c r="DJ1" s="2"/>
-      <c r="DK1" s="2"/>
-      <c r="DL1" s="2"/>
-      <c r="DM1" s="2"/>
-      <c r="DN1" s="2"/>
-      <c r="DO1" s="2"/>
-      <c r="DP1" s="2"/>
-      <c r="DQ1" s="2"/>
-      <c r="DR1" s="1" t="s">
+      <c r="DI1" s="3"/>
+      <c r="DJ1" s="3"/>
+      <c r="DK1" s="3"/>
+      <c r="DL1" s="3"/>
+      <c r="DM1" s="3"/>
+      <c r="DN1" s="3"/>
+      <c r="DO1" s="3"/>
+      <c r="DP1" s="3"/>
+      <c r="DQ1" s="3"/>
+      <c r="DR1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="DS1" s="2"/>
-      <c r="DT1" s="2"/>
-      <c r="DU1" s="2"/>
-      <c r="DV1" s="2"/>
-      <c r="DW1" s="2"/>
-      <c r="DX1" s="2"/>
-      <c r="DY1" s="2"/>
-      <c r="DZ1" s="2"/>
-      <c r="EA1" s="2"/>
-      <c r="EB1" s="1" t="s">
+      <c r="DS1" s="3"/>
+      <c r="DT1" s="3"/>
+      <c r="DU1" s="3"/>
+      <c r="DV1" s="3"/>
+      <c r="DW1" s="3"/>
+      <c r="DX1" s="3"/>
+      <c r="DY1" s="3"/>
+      <c r="DZ1" s="3"/>
+      <c r="EA1" s="3"/>
+      <c r="EB1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="EC1" s="2"/>
-      <c r="ED1" s="2"/>
-      <c r="EE1" s="2"/>
-      <c r="EF1" s="2"/>
-      <c r="EG1" s="2"/>
-      <c r="EH1" s="2"/>
-      <c r="EI1" s="2"/>
-      <c r="EJ1" s="2"/>
-      <c r="EK1" s="2"/>
-      <c r="EL1" s="1" t="s">
+      <c r="EC1" s="3"/>
+      <c r="ED1" s="3"/>
+      <c r="EE1" s="3"/>
+      <c r="EF1" s="3"/>
+      <c r="EG1" s="3"/>
+      <c r="EH1" s="3"/>
+      <c r="EI1" s="3"/>
+      <c r="EJ1" s="3"/>
+      <c r="EK1" s="3"/>
+      <c r="EL1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="EM1" s="2"/>
-      <c r="EN1" s="2"/>
-      <c r="EO1" s="2"/>
-      <c r="EP1" s="2"/>
-      <c r="EQ1" s="2"/>
-      <c r="ER1" s="2"/>
-      <c r="ES1" s="2"/>
-      <c r="ET1" s="2"/>
-      <c r="EU1" s="2"/>
-      <c r="EV1" s="1" t="s">
+      <c r="EM1" s="3"/>
+      <c r="EN1" s="3"/>
+      <c r="EO1" s="3"/>
+      <c r="EP1" s="3"/>
+      <c r="EQ1" s="3"/>
+      <c r="ER1" s="3"/>
+      <c r="ES1" s="3"/>
+      <c r="ET1" s="3"/>
+      <c r="EU1" s="3"/>
+      <c r="EV1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="EW1" s="2"/>
-      <c r="EX1" s="2"/>
-      <c r="EY1" s="2"/>
-      <c r="EZ1" s="2"/>
-      <c r="FA1" s="2"/>
-      <c r="FB1" s="2"/>
-      <c r="FC1" s="2"/>
-      <c r="FD1" s="2"/>
-      <c r="FE1" s="2"/>
+      <c r="EW1" s="3"/>
+      <c r="EX1" s="3"/>
+      <c r="EY1" s="3"/>
+      <c r="EZ1" s="3"/>
+      <c r="FA1" s="3"/>
+      <c r="FB1" s="3"/>
+      <c r="FC1" s="3"/>
+      <c r="FD1" s="3"/>
+      <c r="FE1" s="3"/>
     </row>
     <row r="2" spans="1:161" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
+      <c r="A2" s="3"/>
       <c r="B2" t="s">
         <v>27</v>
       </c>
@@ -6076,6 +6178,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="L1:U1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="EL1:EU1"/>
+    <mergeCell ref="EB1:EK1"/>
+    <mergeCell ref="B1:K1"/>
     <mergeCell ref="EV1:FE1"/>
     <mergeCell ref="V1:AE1"/>
     <mergeCell ref="AF1:AO1"/>
@@ -6088,11 +6195,6 @@
     <mergeCell ref="BT1:CC1"/>
     <mergeCell ref="AP1:AY1"/>
     <mergeCell ref="BJ1:BS1"/>
-    <mergeCell ref="L1:U1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="EL1:EU1"/>
-    <mergeCell ref="EB1:EK1"/>
-    <mergeCell ref="B1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>